<commit_message>
Daily NSE scan: 2026-09-23
</commit_message>
<xml_diff>
--- a/output/2026-09-23/enriched_analysis.xlsx
+++ b/output/2026-09-23/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.674</v>
+        <v>3.54</v>
       </c>
       <c r="W2" t="n">
-        <v>2883</v>
+        <v>2992</v>
       </c>
       <c r="X2" t="n">
-        <v>22.6</v>
+        <v>23.4</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.05</v>
+        <v>0.051</v>
       </c>
       <c r="W3" t="n">
-        <v>2633</v>
+        <v>2620</v>
       </c>
       <c r="X3" t="n">
-        <v>9.050000000000001</v>
+        <v>9.01</v>
       </c>
       <c r="Y3" t="n">
         <v>36</v>
@@ -1399,7 +1399,7 @@
         <v>210</v>
       </c>
       <c r="X4" t="n">
-        <v>8.92</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="Y4" t="n">
         <v>17</v>
@@ -1625,10 +1625,10 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="W5" t="n">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="n">
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.383</v>
+        <v>0.374</v>
       </c>
       <c r="W6" t="n">
-        <v>1225</v>
+        <v>1254</v>
       </c>
       <c r="X6" t="n">
-        <v>62.4</v>
+        <v>63.9</v>
       </c>
       <c r="Y6" t="n">
         <v>21</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.055</v>
+        <v>0.054</v>
       </c>
       <c r="W7" t="n">
-        <v>1507</v>
+        <v>1531</v>
       </c>
       <c r="X7" t="n">
-        <v>20.3</v>
+        <v>20.6</v>
       </c>
       <c r="Y7" t="n">
         <v>55</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.569</v>
       </c>
       <c r="W8" t="n">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="X8" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Y8" t="n">
         <v>22</v>
@@ -2551,10 +2551,10 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.298</v>
+        <v>0.299</v>
       </c>
       <c r="W9" t="n">
-        <v>1029</v>
+        <v>1025</v>
       </c>
       <c r="X9" t="n">
         <v>10.1</v>
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.116</v>
+        <v>0.12</v>
       </c>
       <c r="W10" t="n">
-        <v>2704</v>
+        <v>2625</v>
       </c>
       <c r="X10" t="n">
-        <v>23.7</v>
+        <v>23</v>
       </c>
       <c r="Y10" t="n">
         <v>-3</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.361</v>
+        <v>0.358</v>
       </c>
       <c r="W11" t="n">
-        <v>2691</v>
+        <v>2713</v>
       </c>
       <c r="X11" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="Y11" t="n">
         <v>8</v>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>2.284</v>
+        <v>2.272</v>
       </c>
       <c r="W12" t="n">
-        <v>2609</v>
+        <v>2622</v>
       </c>
       <c r="X12" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Y12" t="n">
         <v>6</v>
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.045</v>
+        <v>0.044</v>
       </c>
       <c r="W13" t="n">
-        <v>15912</v>
+        <v>16554</v>
       </c>
       <c r="X13" t="n">
-        <v>40.5</v>
+        <v>42.2</v>
       </c>
       <c r="Y13" t="n">
         <v>83</v>
@@ -3711,10 +3711,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>1.636</v>
+        <v>1.585</v>
       </c>
       <c r="W14" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="n">
@@ -3941,13 +3941,13 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>0.158</v>
+        <v>0.159</v>
       </c>
       <c r="W15" t="n">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="X15" t="n">
-        <v>58.5</v>
+        <v>58.4</v>
       </c>
       <c r="Y15" t="n">
         <v>3</v>
@@ -4173,13 +4173,13 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.099</v>
+        <v>0.098</v>
       </c>
       <c r="W16" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="X16" t="n">
-        <v>27.8</v>
+        <v>27.9</v>
       </c>
       <c r="Y16" t="n">
         <v>24</v>
@@ -4405,13 +4405,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.077</v>
+        <v>0.076</v>
       </c>
       <c r="W17" t="n">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="X17" t="n">
-        <v>12.9</v>
+        <v>13.1</v>
       </c>
       <c r="Y17" t="n">
         <v>-8</v>
@@ -4637,13 +4637,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="W18" t="n">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="X18" t="n">
-        <v>20.2</v>
+        <v>20.5</v>
       </c>
       <c r="Y18" t="n">
         <v>19</v>
@@ -4867,13 +4867,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>2.338</v>
+        <v>2.305</v>
       </c>
       <c r="W19" t="n">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="X19" t="n">
-        <v>25.6</v>
+        <v>26</v>
       </c>
       <c r="Y19" t="n">
         <v>30</v>
@@ -5093,13 +5093,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.443</v>
+        <v>0.436</v>
       </c>
       <c r="W20" t="n">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="X20" t="n">
-        <v>38.9</v>
+        <v>39.5</v>
       </c>
       <c r="Y20" t="n">
         <v>21</v>
@@ -5325,13 +5325,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.29</v>
+        <v>0.291</v>
       </c>
       <c r="W21" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="X21" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="Y21" t="n">
         <v>12</v>
@@ -5560,10 +5560,10 @@
         <v>0.007</v>
       </c>
       <c r="W22" t="n">
-        <v>5529</v>
+        <v>5550</v>
       </c>
       <c r="X22" t="n">
-        <v>9.34</v>
+        <v>9.4</v>
       </c>
       <c r="Y22" t="n">
         <v>43</v>
@@ -5789,10 +5789,10 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="W23" t="n">
-        <v>990</v>
+        <v>1077</v>
       </c>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="n">
@@ -6022,10 +6022,10 @@
         <v>0.056</v>
       </c>
       <c r="W24" t="n">
-        <v>1977</v>
+        <v>1954</v>
       </c>
       <c r="X24" t="n">
-        <v>45.4</v>
+        <v>44.9</v>
       </c>
       <c r="Y24" t="n">
         <v>20</v>
@@ -6251,13 +6251,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="W25" t="n">
-        <v>5007</v>
+        <v>5056</v>
       </c>
       <c r="X25" t="n">
-        <v>32.6</v>
+        <v>32.9</v>
       </c>
       <c r="Y25" t="n">
         <v>-25</v>
@@ -6275,7 +6275,7 @@
         <v>10.7</v>
       </c>
       <c r="AD25" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AE25" t="b">
         <v>1</v>
@@ -6483,13 +6483,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.038</v>
+        <v>0.036</v>
       </c>
       <c r="W26" t="n">
-        <v>1094</v>
+        <v>1148</v>
       </c>
       <c r="X26" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="Y26" t="n">
         <v>15</v>
@@ -6715,13 +6715,13 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.877</v>
+        <v>0.806</v>
       </c>
       <c r="W27" t="n">
-        <v>226</v>
+        <v>246</v>
       </c>
       <c r="X27" t="n">
-        <v>6.61</v>
+        <v>7.19</v>
       </c>
       <c r="Y27" t="n">
         <v>31</v>
@@ -6943,13 +6943,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.136</v>
+        <v>0.134</v>
       </c>
       <c r="W28" t="n">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="X28" t="n">
-        <v>5.88</v>
+        <v>5.98</v>
       </c>
       <c r="Y28" t="n">
         <v>118</v>
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.533</v>
+        <v>0.529</v>
       </c>
       <c r="W29" t="n">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="X29" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="Y29" t="n">
         <v>19</v>
@@ -7406,7 +7406,7 @@
         <v>0.096</v>
       </c>
       <c r="W30" t="n">
-        <v>1547</v>
+        <v>1546</v>
       </c>
       <c r="X30" t="n">
         <v>14</v>
@@ -7638,10 +7638,10 @@
         <v>0.038</v>
       </c>
       <c r="W31" t="n">
-        <v>3529</v>
+        <v>3550</v>
       </c>
       <c r="X31" t="n">
-        <v>20.9</v>
+        <v>21</v>
       </c>
       <c r="Y31" t="n">
         <v>-4</v>
@@ -7795,16 +7795,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BERGEPAINT</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BERGER PAINTS (I) LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -7812,40 +7812,40 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G32" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>452.6</v>
+        <v>166.59</v>
       </c>
       <c r="J32" t="n">
-        <v>489.56</v>
+        <v>185.61</v>
       </c>
       <c r="K32" t="n">
-        <v>-7.5</v>
+        <v>-10.2</v>
       </c>
       <c r="L32" t="n">
-        <v>75</v>
+        <v>64.08</v>
       </c>
       <c r="M32" t="n">
-        <v>4.84</v>
+        <v>2.4</v>
       </c>
       <c r="N32" t="n">
-        <v>48436318</v>
+        <v>23998951</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>48436318</v>
+        <v>23998951</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -7859,36 +7859,36 @@
         <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="W32" t="n">
-        <v>52773</v>
+        <v>666</v>
       </c>
       <c r="X32" t="n">
-        <v>44.7</v>
+        <v>14.7</v>
       </c>
       <c r="Y32" t="n">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="Z32" t="n">
-        <v>562</v>
+        <v>21</v>
       </c>
       <c r="AA32" t="n">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="AB32" t="n">
-        <v>3.16</v>
+        <v>3.1</v>
       </c>
       <c r="AC32" t="n">
-        <v>22.9</v>
+        <v>19.3</v>
       </c>
       <c r="AD32" t="n">
         <v>0.07000000000000001</v>
@@ -7897,22 +7897,22 @@
         <v>1</v>
       </c>
       <c r="AF32" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="AG32" t="n">
-        <v>502.89</v>
+        <v>168.87</v>
       </c>
       <c r="AH32" t="n">
-        <v>493.7</v>
+        <v>191.99</v>
       </c>
       <c r="AI32" t="n">
-        <v>9.1</v>
+        <v>-2.1</v>
       </c>
       <c r="AJ32" t="n">
-        <v>489.5623319654733</v>
+        <v>185.6067362722351</v>
       </c>
       <c r="AK32" t="n">
-        <v>-7.6</v>
+        <v>-10.2</v>
       </c>
       <c r="AL32" t="inlineStr">
         <is>
@@ -7931,22 +7931,22 @@
       </c>
       <c r="AO32" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="AQ32" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="AR32" t="n">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="AS32" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="AT32" t="n">
         <v>0</v>
@@ -7955,13 +7955,13 @@
         <v>0</v>
       </c>
       <c r="AV32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AW32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AX32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY32" t="n">
         <v>0</v>
@@ -7970,13 +7970,13 @@
         <v>0</v>
       </c>
       <c r="BA32" t="n">
-        <v>48436318</v>
+        <v>8001009</v>
       </c>
       <c r="BB32" t="n">
-        <v>48436318</v>
+        <v>8001009</v>
       </c>
       <c r="BC32" t="n">
-        <v>48436318</v>
+        <v>13998476</v>
       </c>
       <c r="BD32" t="n">
         <v>0</v>
@@ -8012,10 +8012,10 @@
         <v>0</v>
       </c>
       <c r="BO32" t="n">
-        <v>48436318</v>
+        <v>8001009</v>
       </c>
       <c r="BP32" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BQ32" t="n">
         <v>0</v>
@@ -8027,12 +8027,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>BERGEPAINT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
+          <t>BERGER PAINTS (I) LIMITED</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -8044,40 +8044,40 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F33" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G33" t="n">
         <v>9</v>
       </c>
       <c r="H33" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>170.77</v>
+        <v>452.6</v>
       </c>
       <c r="J33" t="n">
-        <v>166.77</v>
+        <v>489.56</v>
       </c>
       <c r="K33" t="n">
-        <v>2.4</v>
+        <v>-7.5</v>
       </c>
       <c r="L33" t="n">
-        <v>61.48</v>
+        <v>75</v>
       </c>
       <c r="M33" t="n">
-        <v>0.4</v>
+        <v>4.84</v>
       </c>
       <c r="N33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -8091,124 +8091,124 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.197</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="W33" t="n">
-        <v>202</v>
+        <v>53601</v>
       </c>
       <c r="X33" t="n">
-        <v>35.1</v>
+        <v>45.4</v>
       </c>
       <c r="Y33" t="n">
-        <v>-44</v>
+        <v>5</v>
       </c>
       <c r="Z33" t="n">
-        <v>-3.28</v>
+        <v>562</v>
       </c>
       <c r="AA33" t="n">
-        <v>141</v>
+        <v>8</v>
       </c>
       <c r="AB33" t="n">
-        <v>-4.05</v>
+        <v>3.16</v>
       </c>
       <c r="AC33" t="n">
-        <v>8.25</v>
+        <v>22.9</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.44</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AE33" t="b">
         <v>1</v>
       </c>
       <c r="AF33" t="n">
-        <v>-35.96</v>
+        <v>17</v>
       </c>
       <c r="AG33" t="n">
-        <v>175.91</v>
+        <v>502.89</v>
       </c>
       <c r="AH33" t="n">
-        <v>179.71</v>
+        <v>493.7</v>
       </c>
       <c r="AI33" t="n">
-        <v>12.7</v>
+        <v>9.1</v>
       </c>
       <c r="AJ33" t="n">
-        <v>166.7666443626631</v>
+        <v>489.5623319654733</v>
       </c>
       <c r="AK33" t="n">
-        <v>2.4</v>
+        <v>-7.6</v>
       </c>
       <c r="AL33" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM33" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN33" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO33" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="AQ33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR33" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="AS33" t="n">
+        <v>16</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
         <v>5</v>
       </c>
-      <c r="AT33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>4</v>
-      </c>
-      <c r="AV33" t="n">
-        <v>4</v>
-      </c>
       <c r="AW33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AX33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AY33" t="n">
-        <v>2606018</v>
+        <v>0</v>
       </c>
       <c r="AZ33" t="n">
-        <v>3987724</v>
+        <v>0</v>
       </c>
       <c r="BA33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="BB33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="BC33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="BD33" t="n">
         <v>0</v>
@@ -8241,75 +8241,75 @@
         <v>0</v>
       </c>
       <c r="BN33" t="n">
-        <v>2606018</v>
+        <v>0</v>
       </c>
       <c r="BO33" t="n">
-        <v>3987724</v>
+        <v>48436318</v>
       </c>
       <c r="BP33" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BQ33" t="n">
         <v>0</v>
       </c>
       <c r="BR33" t="n">
-        <v>0.6535</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Avoid</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I34" t="n">
-        <v>166.59</v>
+        <v>170.77</v>
       </c>
       <c r="J34" t="n">
-        <v>185.61</v>
+        <v>166.77</v>
       </c>
       <c r="K34" t="n">
-        <v>-10.2</v>
+        <v>2.4</v>
       </c>
       <c r="L34" t="n">
-        <v>64.08</v>
+        <v>61.48</v>
       </c>
       <c r="M34" t="n">
-        <v>2.4</v>
+        <v>0.4</v>
       </c>
       <c r="N34" t="n">
-        <v>23998951</v>
+        <v>3987724</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>23998951</v>
+        <v>3987724</v>
       </c>
       <c r="Q34" t="n">
         <v>0</v>
@@ -8327,120 +8327,120 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.357</v>
+        <v>0.195</v>
       </c>
       <c r="W34" t="n">
-        <v>673</v>
+        <v>205</v>
       </c>
       <c r="X34" t="n">
-        <v>14.8</v>
+        <v>35.6</v>
       </c>
       <c r="Y34" t="n">
-        <v>-1</v>
+        <v>-44</v>
       </c>
       <c r="Z34" t="n">
-        <v>21</v>
+        <v>-3.28</v>
       </c>
       <c r="AA34" t="n">
-        <v>45</v>
+        <v>141</v>
       </c>
       <c r="AB34" t="n">
-        <v>3.1</v>
+        <v>-4.05</v>
       </c>
       <c r="AC34" t="n">
-        <v>19.3</v>
+        <v>8.25</v>
       </c>
       <c r="AD34" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="AE34" t="b">
         <v>1</v>
       </c>
       <c r="AF34" t="n">
-        <v>11</v>
+        <v>-35.96</v>
       </c>
       <c r="AG34" t="n">
-        <v>168.87</v>
+        <v>175.91</v>
       </c>
       <c r="AH34" t="n">
-        <v>191.99</v>
+        <v>179.71</v>
       </c>
       <c r="AI34" t="n">
-        <v>-2.1</v>
+        <v>12.7</v>
       </c>
       <c r="AJ34" t="n">
-        <v>185.6067362722351</v>
+        <v>166.7666443626631</v>
       </c>
       <c r="AK34" t="n">
-        <v>-10.2</v>
+        <v>2.4</v>
       </c>
       <c r="AL34" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM34" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN34" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO34" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="AQ34" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="AR34" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="AS34" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="AT34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AW34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AY34" t="n">
-        <v>0</v>
+        <v>2606018</v>
       </c>
       <c r="AZ34" t="n">
-        <v>0</v>
+        <v>3987724</v>
       </c>
       <c r="BA34" t="n">
-        <v>8001009</v>
+        <v>3987724</v>
       </c>
       <c r="BB34" t="n">
-        <v>8001009</v>
+        <v>3987724</v>
       </c>
       <c r="BC34" t="n">
-        <v>13998476</v>
+        <v>3987724</v>
       </c>
       <c r="BD34" t="n">
         <v>0</v>
@@ -8473,10 +8473,10 @@
         <v>0</v>
       </c>
       <c r="BN34" t="n">
-        <v>0</v>
+        <v>2606018</v>
       </c>
       <c r="BO34" t="n">
-        <v>8001009</v>
+        <v>3987724</v>
       </c>
       <c r="BP34" t="n">
         <v>1</v>
@@ -8485,7 +8485,7 @@
         <v>0</v>
       </c>
       <c r="BR34" t="n">
-        <v>0</v>
+        <v>0.6535</v>
       </c>
     </row>
     <row r="35">
@@ -8563,13 +8563,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.074</v>
       </c>
       <c r="W35" t="n">
-        <v>743</v>
+        <v>731</v>
       </c>
       <c r="X35" t="n">
-        <v>13.5</v>
+        <v>13.3</v>
       </c>
       <c r="Y35" t="n">
         <v>185</v>
@@ -8793,13 +8793,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.646</v>
+        <v>0.626</v>
       </c>
       <c r="W36" t="n">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="X36" t="n">
-        <v>1172</v>
+        <v>1211</v>
       </c>
       <c r="Y36" t="n">
         <v>-61</v>
@@ -9024,10 +9024,10 @@
         <v>0.021</v>
       </c>
       <c r="W37" t="n">
-        <v>9344</v>
+        <v>9468</v>
       </c>
       <c r="X37" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="Y37" t="n">
         <v>-12</v>
@@ -9256,10 +9256,10 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>3941</v>
+        <v>3857</v>
       </c>
       <c r="X38" t="n">
-        <v>88.7</v>
+        <v>86.8</v>
       </c>
       <c r="Y38" t="n">
         <v>42</v>
@@ -9488,10 +9488,10 @@
         <v>0.128</v>
       </c>
       <c r="W39" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="X39" t="n">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
       <c r="Y39" t="n">
         <v>61</v>
@@ -9715,13 +9715,13 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.544</v>
+        <v>0.54</v>
       </c>
       <c r="W40" t="n">
-        <v>3554</v>
+        <v>3580</v>
       </c>
       <c r="X40" t="n">
-        <v>24.9</v>
+        <v>25.1</v>
       </c>
       <c r="Y40" t="n">
         <v>2</v>
@@ -9950,10 +9950,10 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="X41" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="Y41" t="n">
         <v>5</v>
@@ -10179,13 +10179,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.207</v>
+        <v>0.211</v>
       </c>
       <c r="W42" t="n">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="X42" t="n">
-        <v>25.8</v>
+        <v>25.4</v>
       </c>
       <c r="Y42" t="n">
         <v>21</v>
@@ -10411,13 +10411,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.224</v>
+        <v>0.221</v>
       </c>
       <c r="W43" t="n">
-        <v>1783</v>
+        <v>1809</v>
       </c>
       <c r="X43" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="Y43" t="n">
         <v>-3</v>
@@ -10646,10 +10646,10 @@
         <v>0.042</v>
       </c>
       <c r="W44" t="n">
-        <v>1659</v>
+        <v>1639</v>
       </c>
       <c r="X44" t="n">
-        <v>21.7</v>
+        <v>21.4</v>
       </c>
       <c r="Y44" t="n">
         <v>10</v>
@@ -10875,13 +10875,13 @@
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.232</v>
+        <v>0.226</v>
       </c>
       <c r="W45" t="n">
-        <v>970</v>
+        <v>996</v>
       </c>
       <c r="X45" t="n">
-        <v>26.4</v>
+        <v>27.1</v>
       </c>
       <c r="Y45" t="n">
         <v>9</v>
@@ -11107,13 +11107,13 @@
         </is>
       </c>
       <c r="V46" t="n">
-        <v>0.35</v>
+        <v>0.343</v>
       </c>
       <c r="W46" t="n">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="X46" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="Y46" t="n">
         <v>246</v>
@@ -11342,10 +11342,10 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>2330</v>
+        <v>2543</v>
       </c>
       <c r="X47" t="n">
-        <v>689</v>
+        <v>752</v>
       </c>
       <c r="Y47" t="n">
         <v>3</v>
@@ -11574,10 +11574,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>8907</v>
+        <v>9117</v>
       </c>
       <c r="X48" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
@@ -12038,10 +12038,10 @@
         <v>0</v>
       </c>
       <c r="W50" t="n">
-        <v>116392</v>
+        <v>119952</v>
       </c>
       <c r="X50" t="n">
-        <v>33.5</v>
+        <v>34.5</v>
       </c>
       <c r="Y50" t="n">
         <v>18</v>
@@ -12267,13 +12267,13 @@
         </is>
       </c>
       <c r="V51" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
       <c r="W51" t="n">
-        <v>1670</v>
+        <v>1699</v>
       </c>
       <c r="X51" t="n">
-        <v>30.1</v>
+        <v>30.7</v>
       </c>
       <c r="Y51" t="n">
         <v>39</v>
@@ -13549,105 +13549,105 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BERGEPAINT</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BERGER PAINTS (I) LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>452.6</v>
+        <v>166.59</v>
       </c>
       <c r="D32" t="n">
-        <v>489.56</v>
+        <v>185.61</v>
       </c>
       <c r="E32" t="n">
-        <v>-7.5</v>
+        <v>-10.2</v>
       </c>
       <c r="F32" t="n">
-        <v>75</v>
+        <v>64.08</v>
       </c>
       <c r="G32" t="n">
-        <v>4.84</v>
+        <v>2.4</v>
       </c>
       <c r="H32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>BERGEPAINT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
+          <t>BERGER PAINTS (I) LIMITED</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>170.77</v>
+        <v>452.6</v>
       </c>
       <c r="D33" t="n">
-        <v>166.77</v>
+        <v>489.56</v>
       </c>
       <c r="E33" t="n">
-        <v>2.4</v>
+        <v>-7.5</v>
       </c>
       <c r="F33" t="n">
-        <v>61.48</v>
+        <v>75</v>
       </c>
       <c r="G33" t="n">
-        <v>0.4</v>
+        <v>4.84</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>166.59</v>
+        <v>170.77</v>
       </c>
       <c r="D34" t="n">
-        <v>185.61</v>
+        <v>166.77</v>
       </c>
       <c r="E34" t="n">
-        <v>-10.2</v>
+        <v>2.4</v>
       </c>
       <c r="F34" t="n">
-        <v>64.08</v>
+        <v>61.48</v>
       </c>
       <c r="G34" t="n">
-        <v>2.4</v>
+        <v>0.4</v>
       </c>
       <c r="H34" t="n">
         <v>4</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
     </row>
@@ -14329,7 +14329,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -14349,7 +14349,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">

</xml_diff>